<commit_message>
Switch Elkanah Part Fees to residual formula; add & highlight H test cells
- F15 (Cashout) / F17 (Card Transfer): replace flat-cap Part Fees text
  with the residual definition (Total - SLP - Cashback), reconciling the
  caps that previously did not balance at large amounts. Express Revenue
  as (Part Fees - ISW)*100/107.5 and VAT as 7.5% of Revenue so the
  breakdown ties out at every transaction size.
- Add residual formula to the Part Fees test-value cells
  (H15 = -H12-H13-H14; H17 = -H14-H15-H16) plus the Silver cashback
  cells they reference (H14/H16 = 0), and highlight these cells yellow.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KLEDw2XETUjv47sCErMpSv
</commit_message>
<xml_diff>
--- a/Updated_Agent_User_Accounting_Schematics_EMTL_ISW_VATincl (updated).xlsx
+++ b/Updated_Agent_User_Accounting_Schematics_EMTL_ISW_VATincl (updated).xlsx
@@ -1802,7 +1802,7 @@
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="795">
+  <cellXfs count="797">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -3504,6 +3504,8 @@
     <xf numFmtId="177" fontId="15" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="2" fontId="9" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="2" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5148,7 +5150,9 @@
 IF (Platinum Agent, cashback = (0.001 * Nxxx capped at N20.00)</t>
         </is>
       </c>
-      <c r="H14" s="368" t="n"/>
+      <c r="H14" s="795" t="n">
+        <v>0</v>
+      </c>
       <c r="J14" s="728" t="n"/>
     </row>
     <row r="15" ht="41" customHeight="1" s="581" thickBot="1">
@@ -5174,15 +5178,19 @@
       </c>
       <c r="F15" s="729" t="inlineStr">
         <is>
-          <t>Part Fees to Elkanah Suspense (= ISW + Revenue to 9PSB + VAT on revenue).
-IF (Silver Agent = 0.00460 * Nxxx, capped at N75.00)
-IF (Gold Agent = 0.00410 * Nxxx, capped at N65.00)
-IF (Platinum Agent = 0.00360 * Nxxx, capped at N55.00)
-Derivation / breakdown of Part Fees (the portion 9PSB keeps = Revenue + VAT; the ISW fee is settled on the Core Banking System and therefore does NOT reflect as 9PSB income here):
-  - ISW (settled on Core Banking): 0.003225 * Nxxx (capped at N21.50)
-  - Revenue to 9PSB: Silver 0.00127907 (cap N65.58) | Gold 0.000813953 (cap N56.28) | Platinum 0.000348837 (cap N46.98)
-  - VAT on revenue: Silver 0.0000959302 (cap N4.92) | Gold 0.0000610465 (cap N4.22) | Platinum 0.0000261628 (cap N3.52)</t>
-        </is>
+          <t>Part Fees to Elkanah Suspense = Total Charge - SLP - Cashback  (the residual).
+= ISW + Revenue to 9PSB + VAT on revenue.
+  Uncapped portion: Silver 0.0046 x Nxxx | Gold 0.0041 x Nxxx | Platinum 0.0036 x Nxxx.
+  Effective ceiling at large amounts (Total, SLP &amp; ISW each capped): Silver N75.00 | Gold N65.00 | Platinum N55.00.
+9PSB keeps Revenue + VAT; the ISW fee is settled on the Core Banking System and does NOT reflect as 9PSB income here:
+  - ISW (settled on Core Banking): 0.003225 x Nxxx (capped at N21.50)
+  - Revenue to 9PSB = (Part Fees - ISW) x 100/107.5
+  - VAT on revenue  = 7.5% x Revenue</t>
+        </is>
+      </c>
+      <c r="H15" s="796">
+        <f>-H12-H13-H14</f>
+        <v/>
       </c>
       <c r="I15" s="730" t="n"/>
     </row>
@@ -6003,7 +6011,9 @@
 IF (Platinum Agent, cashback = (0.001 * Nxxx capped at N20.00)</t>
         </is>
       </c>
-      <c r="H16" s="368" t="n"/>
+      <c r="H16" s="795" t="n">
+        <v>0</v>
+      </c>
       <c r="J16" s="728" t="n"/>
     </row>
     <row r="17" ht="41" customHeight="1" s="581" thickBot="1">
@@ -6029,15 +6039,19 @@
       </c>
       <c r="F17" s="729" t="inlineStr">
         <is>
-          <t>Part Fees to Elkanah Suspense (= ISW + Revenue to 9PSB + VAT on revenue).
-IF (Silver Agent = 0.00460 * Nxxx, capped at N75.00)
-IF (Gold Agent = 0.00410 * Nxxx, capped at N65.00)
-IF (Platinum Agent = 0.00360 * Nxxx, capped at N55.00)
-Derivation / breakdown of Part Fees (the portion 9PSB keeps = Revenue + VAT; the ISW fee is settled on the Core Banking System and therefore does NOT reflect as 9PSB income here):
-  - ISW (settled on Core Banking): 0.003225 * Nxxx (capped at N21.50)
-  - Revenue to 9PSB: Silver 0.00127907 (cap N65.58) | Gold 0.000813953 (cap N56.28) | Platinum 0.000348837 (cap N46.98)
-  - VAT on revenue: Silver 0.0000959302 (cap N4.92) | Gold 0.0000610465 (cap N4.22) | Platinum 0.0000261628 (cap N3.52)</t>
-        </is>
+          <t>Part Fees to Elkanah Suspense = Total Charge - SLP - Cashback  (the residual).
+= ISW + Revenue to 9PSB + VAT on revenue.
+  Uncapped portion: Silver 0.0046 x Nxxx | Gold 0.0041 x Nxxx | Platinum 0.0036 x Nxxx.
+  Effective ceiling at large amounts (Total, SLP &amp; ISW each capped): Silver N75.00 | Gold N65.00 | Platinum N55.00.
+9PSB keeps Revenue + VAT; the ISW fee is settled on the Core Banking System and does NOT reflect as 9PSB income here:
+  - ISW (settled on Core Banking): 0.003225 x Nxxx (capped at N21.50)
+  - Revenue to 9PSB = (Part Fees - ISW) x 100/107.5
+  - VAT on revenue  = 7.5% x Revenue</t>
+        </is>
+      </c>
+      <c r="H17" s="796">
+        <f>-H14-H15-H16</f>
+        <v/>
       </c>
       <c r="I17" s="730" t="n"/>
     </row>

</xml_diff>

<commit_message>
Reconcile core-banking Revenue/VAT caps to the Part Fees pot ceiling
The core-banking 9PSB Revenue/VAT caps were computed on a different
transaction size (N20,000, SLP=8) than the Elkanah Part Fees ceilings
(N75/65/55, which use SLP fully capped at N25), so they did not tie out.
Reset them from the pot: pool = ceiling - ISW(21.50); Revenue = pool*100/107.5,
VAT = pool*7.5/107.5.

- Silver: Revenue 65.58->49.77, VAT 4.92->3.73 (pot 75)
- Gold:   Revenue 56.28->40.47, VAT 4.22->3.03 (pot 65)
- Platinum: Revenue 46.98->31.16, VAT 3.52->2.34 (pot 55)

Updated F/H cells on Cashout with Card (ISW) and Card Transfer (ISW);
highlighted the changed H cap cells. Splitting tabs unaffected (already
residual-based with no hardcoded caps).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KLEDw2XETUjv47sCErMpSv
</commit_message>
<xml_diff>
--- a/Updated_Agent_User_Accounting_Schematics_EMTL_ISW_VATincl (updated).xlsx
+++ b/Updated_Agent_User_Accounting_Schematics_EMTL_ISW_VATincl (updated).xlsx
@@ -5369,13 +5369,13 @@
       </c>
       <c r="F26" s="490" t="inlineStr">
         <is>
-          <t>IF (Silver Agent = 0.00127907 * Nxxx capped at N65.58), 
-IF (Gold Agent = 0.000813953 * Nxxx capped at N56.28), 
-IF (Platinum Agent = 0.000348837 * Nxxx capped at N46.98)</t>
+          <t>IF (Silver Agent = 0.00127907 * Nxxx capped at N49.77), 
+IF (Gold Agent = 0.000813953 * Nxxx capped at N40.47), 
+IF (Platinum Agent = 0.000348837 * Nxxx capped at N31.16)</t>
         </is>
       </c>
       <c r="H26" s="491">
-        <f>IF(0.00127907*H19&gt;65.58,65.58,0.00127907*H19)</f>
+        <f>IF(0.00127907*H19&gt;49.77,49.77,0.00127907*H19)</f>
         <v/>
       </c>
       <c r="J26" s="281">
@@ -5404,13 +5404,13 @@
       </c>
       <c r="F27" s="490" t="inlineStr">
         <is>
-          <t>IF (Silver Agent = 0.0000959302 * Nxxx capped at N4.92 ), 
-IF (Gold Agent = 0.0000610465 * Nxxx capped at N4.22 ), 
-IF (Platinum Agent = 0.0000261628 * Nxxx capped at N3.52)</t>
+          <t>IF (Silver Agent = 0.0000959302 * Nxxx capped at N3.73 ), 
+IF (Gold Agent = 0.0000610465 * Nxxx capped at N3.03 ), 
+IF (Platinum Agent = 0.0000261628 * Nxxx capped at N2.34)</t>
         </is>
       </c>
       <c r="H27" s="491">
-        <f>IF(0.0000959302*H19&gt;4.92,4.92,0.0000959302*H19)</f>
+        <f>IF(0.0000959302*H19&gt;3.73,3.73,0.0000959302*H19)</f>
         <v/>
       </c>
       <c r="J27" s="281">
@@ -6230,13 +6230,13 @@
       </c>
       <c r="F28" s="490" t="inlineStr">
         <is>
-          <t>IF (Silver Agent = 0.00127907 * Nxxx capped at N65.58), 
-IF (Gold Agent = 0.000813953 * Nxxx capped at N56.28), 
-IF (Platinum Agent = 0.000348837 * Nxxx capped at N46.98)</t>
+          <t>IF (Silver Agent = 0.00127907 * Nxxx capped at N49.77), 
+IF (Gold Agent = 0.000813953 * Nxxx capped at N40.47), 
+IF (Platinum Agent = 0.000348837 * Nxxx capped at N31.16)</t>
         </is>
       </c>
       <c r="H28" s="491">
-        <f>IF(0.00127907*H21&gt;65.58,65.58,0.00127907*H21)</f>
+        <f>IF(0.00127907*H21&gt;49.77,49.77,0.00127907*H21)</f>
         <v/>
       </c>
       <c r="J28" s="281">
@@ -6265,13 +6265,13 @@
       </c>
       <c r="F29" s="490" t="inlineStr">
         <is>
-          <t>IF (Silver Agent = 0.0000959302 * Nxxx capped at N4.92 ), 
-IF (Gold Agent = 0.0000610465 * Nxxx capped at N4.22 ), 
-IF (Platinum Agent = 0.0000261628 * Nxxx capped at N3.52)</t>
+          <t>IF (Silver Agent = 0.0000959302 * Nxxx capped at N3.73 ), 
+IF (Gold Agent = 0.0000610465 * Nxxx capped at N3.03 ), 
+IF (Platinum Agent = 0.0000261628 * Nxxx capped at N2.34)</t>
         </is>
       </c>
       <c r="H29" s="491">
-        <f>IF(0.0000959302*H21&gt;4.92,4.92,0.0000959302*H21)</f>
+        <f>IF(0.0000959302*H21&gt;3.73,3.73,0.0000959302*H21)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert core-banking caps (correct) and fix Elkanah Part Fees ceiling to max
Correction: the core-banking Revenue/VAT caps (65.58/56.28/46.98 +
4.92/4.22/3.52) are correct - they are the MAXIMUM, reached at the
N20,000 band where the N100 total cap binds while SLP is still N8. My
earlier change to 49.77 used the >=N62,500 asymptote and was wrong.

- Restored F26/F27/H26/H27 (Cashout) and F28/F29/H28/H29 (Card Transfer)
  to the original 65.58/56.28/46.98 + 4.92/4.22/3.52.
- Fixed the Elkanah Part Fees ceiling 75/65/55 -> 92/82/72 (the true max
  at N20,000), reconciling with core banking: 21.50 + 65.58 + 4.92 = 92.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KLEDw2XETUjv47sCErMpSv
</commit_message>
<xml_diff>
--- a/Updated_Agent_User_Accounting_Schematics_EMTL_ISW_VATincl (updated).xlsx
+++ b/Updated_Agent_User_Accounting_Schematics_EMTL_ISW_VATincl (updated).xlsx
@@ -5178,14 +5178,10 @@
       </c>
       <c r="F15" s="729" t="inlineStr">
         <is>
-          <t>Part Fees to Elkanah Suspense = Total Charge - SLP - Cashback  (the residual).
-= ISW + Revenue to 9PSB + VAT on revenue.
-  Uncapped portion: Silver 0.0046 x Nxxx | Gold 0.0041 x Nxxx | Platinum 0.0036 x Nxxx.
-  Effective ceiling at large amounts (Total, SLP &amp; ISW each capped): Silver N75.00 | Gold N65.00 | Platinum N55.00.
-9PSB keeps Revenue + VAT; the ISW fee is settled on the Core Banking System and does NOT reflect as 9PSB income here:
-  - ISW (settled on Core Banking): 0.003225 x Nxxx (capped at N21.50)
-  - Revenue to 9PSB = (Part Fees - ISW) x 100/107.5
-  - VAT on revenue  = 7.5% x Revenue</t>
+          <t>Part Fees to Elkanah Suspense = Total Charge - SLP - Cashback (residual) -&gt; settled on Core Banking as ISW + Revenue to 9PSB + VAT.
+Silver 0.46% | Gold 0.41% | Platinum 0.36% of Nxxx (up to the N100 total-charge cap).
+Maximum Part Fees (at N20,000, where the N100 total cap binds): Silver N92.00 | Gold N82.00 | Platinum N72.00
+  = ISW N21.50 + Revenue (Silver 65.58 / Gold 56.28 / Platinum 46.98) + VAT (Silver 4.92 / Gold 4.22 / Platinum 3.52).</t>
         </is>
       </c>
       <c r="H15" s="796">
@@ -5369,13 +5365,13 @@
       </c>
       <c r="F26" s="490" t="inlineStr">
         <is>
-          <t>IF (Silver Agent = 0.00127907 * Nxxx capped at N49.77), 
-IF (Gold Agent = 0.000813953 * Nxxx capped at N40.47), 
-IF (Platinum Agent = 0.000348837 * Nxxx capped at N31.16)</t>
+          <t>IF (Silver Agent = 0.00127907 * Nxxx capped at N65.58), 
+IF (Gold Agent = 0.000813953 * Nxxx capped at N56.28), 
+IF (Platinum Agent = 0.000348837 * Nxxx capped at N46.98)</t>
         </is>
       </c>
       <c r="H26" s="491">
-        <f>IF(0.00127907*H19&gt;49.77,49.77,0.00127907*H19)</f>
+        <f>IF(0.00127907*H19&gt;65.58,65.58,0.00127907*H19)</f>
         <v/>
       </c>
       <c r="J26" s="281">
@@ -5404,13 +5400,13 @@
       </c>
       <c r="F27" s="490" t="inlineStr">
         <is>
-          <t>IF (Silver Agent = 0.0000959302 * Nxxx capped at N3.73 ), 
-IF (Gold Agent = 0.0000610465 * Nxxx capped at N3.03 ), 
-IF (Platinum Agent = 0.0000261628 * Nxxx capped at N2.34)</t>
+          <t>IF (Silver Agent = 0.0000959302 * Nxxx capped at N4.92 ), 
+IF (Gold Agent = 0.0000610465 * Nxxx capped at N4.22 ), 
+IF (Platinum Agent = 0.0000261628 * Nxxx capped at N3.52)</t>
         </is>
       </c>
       <c r="H27" s="491">
-        <f>IF(0.0000959302*H19&gt;3.73,3.73,0.0000959302*H19)</f>
+        <f>IF(0.0000959302*H19&gt;4.92,4.92,0.0000959302*H19)</f>
         <v/>
       </c>
       <c r="J27" s="281">
@@ -6039,14 +6035,10 @@
       </c>
       <c r="F17" s="729" t="inlineStr">
         <is>
-          <t>Part Fees to Elkanah Suspense = Total Charge - SLP - Cashback  (the residual).
-= ISW + Revenue to 9PSB + VAT on revenue.
-  Uncapped portion: Silver 0.0046 x Nxxx | Gold 0.0041 x Nxxx | Platinum 0.0036 x Nxxx.
-  Effective ceiling at large amounts (Total, SLP &amp; ISW each capped): Silver N75.00 | Gold N65.00 | Platinum N55.00.
-9PSB keeps Revenue + VAT; the ISW fee is settled on the Core Banking System and does NOT reflect as 9PSB income here:
-  - ISW (settled on Core Banking): 0.003225 x Nxxx (capped at N21.50)
-  - Revenue to 9PSB = (Part Fees - ISW) x 100/107.5
-  - VAT on revenue  = 7.5% x Revenue</t>
+          <t>Part Fees to Elkanah Suspense = Total Charge - SLP - Cashback (residual) -&gt; settled on Core Banking as ISW + Revenue to 9PSB + VAT.
+Silver 0.46% | Gold 0.41% | Platinum 0.36% of Nxxx (up to the N100 total-charge cap).
+Maximum Part Fees (at N20,000, where the N100 total cap binds): Silver N92.00 | Gold N82.00 | Platinum N72.00
+  = ISW N21.50 + Revenue (Silver 65.58 / Gold 56.28 / Platinum 46.98) + VAT (Silver 4.92 / Gold 4.22 / Platinum 3.52).</t>
         </is>
       </c>
       <c r="H17" s="796">
@@ -6230,13 +6222,13 @@
       </c>
       <c r="F28" s="490" t="inlineStr">
         <is>
-          <t>IF (Silver Agent = 0.00127907 * Nxxx capped at N49.77), 
-IF (Gold Agent = 0.000813953 * Nxxx capped at N40.47), 
-IF (Platinum Agent = 0.000348837 * Nxxx capped at N31.16)</t>
+          <t>IF (Silver Agent = 0.00127907 * Nxxx capped at N65.58), 
+IF (Gold Agent = 0.000813953 * Nxxx capped at N56.28), 
+IF (Platinum Agent = 0.000348837 * Nxxx capped at N46.98)</t>
         </is>
       </c>
       <c r="H28" s="491">
-        <f>IF(0.00127907*H21&gt;49.77,49.77,0.00127907*H21)</f>
+        <f>IF(0.00127907*H21&gt;65.58,65.58,0.00127907*H21)</f>
         <v/>
       </c>
       <c r="J28" s="281">
@@ -6265,13 +6257,13 @@
       </c>
       <c r="F29" s="490" t="inlineStr">
         <is>
-          <t>IF (Silver Agent = 0.0000959302 * Nxxx capped at N3.73 ), 
-IF (Gold Agent = 0.0000610465 * Nxxx capped at N3.03 ), 
-IF (Platinum Agent = 0.0000261628 * Nxxx capped at N2.34)</t>
+          <t>IF (Silver Agent = 0.0000959302 * Nxxx capped at N4.92 ), 
+IF (Gold Agent = 0.0000610465 * Nxxx capped at N4.22 ), 
+IF (Platinum Agent = 0.0000261628 * Nxxx capped at N3.52)</t>
         </is>
       </c>
       <c r="H29" s="491">
-        <f>IF(0.0000959302*H21&gt;3.73,3.73,0.0000959302*H21)</f>
+        <f>IF(0.0000959302*H21&gt;4.92,4.92,0.0000959302*H21)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Reformat Elkanah Part Fees to match core-banking per-tier IF style
F15 (Cashout) / F17 (Card Transfer) now read:
  IF (Silver Agent = 0.0046 * Nxxx capped at N92.00),
  IF (Gold Agent   = 0.0041 * Nxxx capped at N82.00),
  IF (Platinum Agent = 0.0036 * Nxxx capped at N72.00)
mirroring the Revenue/VAT line format, with the corrected N92/82/72 caps.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KLEDw2XETUjv47sCErMpSv
</commit_message>
<xml_diff>
--- a/Updated_Agent_User_Accounting_Schematics_EMTL_ISW_VATincl (updated).xlsx
+++ b/Updated_Agent_User_Accounting_Schematics_EMTL_ISW_VATincl (updated).xlsx
@@ -5178,10 +5178,9 @@
       </c>
       <c r="F15" s="729" t="inlineStr">
         <is>
-          <t>Part Fees to Elkanah Suspense = Total Charge - SLP - Cashback (residual) -&gt; settled on Core Banking as ISW + Revenue to 9PSB + VAT.
-Silver 0.46% | Gold 0.41% | Platinum 0.36% of Nxxx (up to the N100 total-charge cap).
-Maximum Part Fees (at N20,000, where the N100 total cap binds): Silver N92.00 | Gold N82.00 | Platinum N72.00
-  = ISW N21.50 + Revenue (Silver 65.58 / Gold 56.28 / Platinum 46.98) + VAT (Silver 4.92 / Gold 4.22 / Platinum 3.52).</t>
+          <t>IF (Silver Agent = 0.0046 * Nxxx capped at N92.00), 
+IF (Gold Agent = 0.0041 * Nxxx capped at N82.00), 
+IF (Platinum Agent = 0.0036 * Nxxx capped at N72.00)</t>
         </is>
       </c>
       <c r="H15" s="796">
@@ -6035,10 +6034,9 @@
       </c>
       <c r="F17" s="729" t="inlineStr">
         <is>
-          <t>Part Fees to Elkanah Suspense = Total Charge - SLP - Cashback (residual) -&gt; settled on Core Banking as ISW + Revenue to 9PSB + VAT.
-Silver 0.46% | Gold 0.41% | Platinum 0.36% of Nxxx (up to the N100 total-charge cap).
-Maximum Part Fees (at N20,000, where the N100 total cap binds): Silver N92.00 | Gold N82.00 | Platinum N72.00
-  = ISW N21.50 + Revenue (Silver 65.58 / Gold 56.28 / Platinum 46.98) + VAT (Silver 4.92 / Gold 4.22 / Platinum 3.52).</t>
+          <t>IF (Silver Agent = 0.0046 * Nxxx capped at N92.00), 
+IF (Gold Agent = 0.0041 * Nxxx capped at N82.00), 
+IF (Platinum Agent = 0.0036 * Nxxx capped at N72.00)</t>
         </is>
       </c>
       <c r="H17" s="796">

</xml_diff>